<commit_message>
Run ulang pipeline: workbook RTOW periodik terupdate + TANJU & MENGKOANG pindah 15 Harian
- data_bon: new_data_bon_a_bon_b_rtow_ketersediaan_kebutuhan_air.xlsx terbaru
  (212 bendungan, 11 sheet, elevasi kekeringan lengkap)
- fromat-rtow.csv: TANJU (302) & MENGKOANG (172) 10 Harian -> 15 Harian
  (model 15H kini 122 bendungan)
- Ekstraksi ulang SINBAD (TMA s.d. 30 Jul 2026), QC lolos 210 bendungan
- Training ulang LSTM 15H & 10H + prediksi Agu-Des 2026 + evaluasi backtest
  (LSTM tetap terbaik: MAE 1,25 m Agu-Des 2025; 0,90 m Mar-Jul 2026)
- run_pipeline.py: print penutup tanpa simbol unicode (crash cp1252 Windows)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/processed/rekap_qc.xlsx
+++ b/data/processed/rekap_qc.xlsx
@@ -5027,7 +5027,7 @@
         <v>180</v>
       </c>
       <c r="B174">
-        <v>2877</v>
+        <v>2876</v>
       </c>
       <c r="C174">
         <v>0</v>
@@ -5036,10 +5036,10 @@
         <v>0</v>
       </c>
       <c r="E174">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="F174">
-        <v>2588</v>
+        <v>2585</v>
       </c>
       <c r="G174" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
update bulan oktober 2026
</commit_message>
<xml_diff>
--- a/data/processed/rekap_qc.xlsx
+++ b/data/processed/rekap_qc.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="221">
   <si>
     <t>kode_bendungan</t>
   </si>
@@ -1071,13 +1071,13 @@
         <v>2544</v>
       </c>
       <c r="C2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F2">
         <v>2527</v>
@@ -1094,13 +1094,13 @@
         <v>2546</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F3">
         <v>2527</v>
@@ -1183,7 +1183,7 @@
         <v>13</v>
       </c>
       <c r="B7">
-        <v>2548</v>
+        <v>2549</v>
       </c>
       <c r="C7">
         <v>2</v>
@@ -1192,7 +1192,7 @@
         <v>0</v>
       </c>
       <c r="E7">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F7">
         <v>2527</v>
@@ -1232,13 +1232,13 @@
         <v>2544</v>
       </c>
       <c r="C9">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D9">
         <v>0</v>
       </c>
       <c r="E9">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F9">
         <v>2527</v>
@@ -1344,7 +1344,7 @@
         <v>20</v>
       </c>
       <c r="B14">
-        <v>2544</v>
+        <v>2549</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -1353,7 +1353,7 @@
         <v>0</v>
       </c>
       <c r="E14">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F14">
         <v>2527</v>
@@ -1462,13 +1462,13 @@
         <v>2545</v>
       </c>
       <c r="C19">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D19">
         <v>0</v>
       </c>
       <c r="E19">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F19">
         <v>2527</v>
@@ -1577,13 +1577,13 @@
         <v>2544</v>
       </c>
       <c r="C24">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E24">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F24">
         <v>2527</v>
@@ -1666,7 +1666,7 @@
         <v>34</v>
       </c>
       <c r="B28">
-        <v>2544</v>
+        <v>2545</v>
       </c>
       <c r="C28">
         <v>2</v>
@@ -1675,7 +1675,7 @@
         <v>0</v>
       </c>
       <c r="E28">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F28">
         <v>2527</v>
@@ -1776,7 +1776,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:7">
       <c r="A33" t="s">
         <v>39</v>
       </c>
@@ -1799,7 +1799,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:7">
       <c r="A34" t="s">
         <v>40</v>
       </c>
@@ -1822,7 +1822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:8">
+    <row r="35" spans="1:7">
       <c r="A35" t="s">
         <v>41</v>
       </c>
@@ -1845,12 +1845,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
+    <row r="36" spans="1:7">
       <c r="A36" t="s">
         <v>42</v>
       </c>
       <c r="B36">
-        <v>2546</v>
+        <v>2547</v>
       </c>
       <c r="C36">
         <v>0</v>
@@ -1859,7 +1859,7 @@
         <v>0</v>
       </c>
       <c r="E36">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F36">
         <v>2527</v>
@@ -1868,7 +1868,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
+    <row r="37" spans="1:7">
       <c r="A37" t="s">
         <v>43</v>
       </c>
@@ -1891,12 +1891,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" spans="1:7">
       <c r="A38" t="s">
         <v>44</v>
       </c>
       <c r="B38">
-        <v>2587</v>
+        <v>2590</v>
       </c>
       <c r="C38">
         <v>0</v>
@@ -1905,7 +1905,7 @@
         <v>0</v>
       </c>
       <c r="E38">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F38">
         <v>2525</v>
@@ -1914,7 +1914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
+    <row r="39" spans="1:7">
       <c r="A39" t="s">
         <v>45</v>
       </c>
@@ -1937,12 +1937,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:8">
+    <row r="40" spans="1:7">
       <c r="A40" t="s">
         <v>46</v>
       </c>
       <c r="B40">
-        <v>2697</v>
+        <v>2698</v>
       </c>
       <c r="C40">
         <v>0</v>
@@ -1951,7 +1951,7 @@
         <v>0</v>
       </c>
       <c r="E40">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F40">
         <v>2566</v>
@@ -1960,7 +1960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:8">
+    <row r="41" spans="1:7">
       <c r="A41" t="s">
         <v>47</v>
       </c>
@@ -1983,7 +1983,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:8">
+    <row r="42" spans="1:7">
       <c r="A42" t="s">
         <v>48</v>
       </c>
@@ -2006,7 +2006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:8">
+    <row r="43" spans="1:7">
       <c r="A43" t="s">
         <v>49</v>
       </c>
@@ -2014,7 +2014,7 @@
         <v>2552</v>
       </c>
       <c r="C43">
-        <v>404</v>
+        <v>434</v>
       </c>
       <c r="D43">
         <v>0</v>
@@ -2023,13 +2023,13 @@
         <v>57</v>
       </c>
       <c r="F43">
-        <v>2899</v>
+        <v>2929</v>
       </c>
       <c r="G43" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:8">
+    <row r="44" spans="1:7">
       <c r="A44" t="s">
         <v>50</v>
       </c>
@@ -2052,7 +2052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:8">
+    <row r="45" spans="1:7">
       <c r="A45" t="s">
         <v>51</v>
       </c>
@@ -2075,7 +2075,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:8">
+    <row r="46" spans="1:7">
       <c r="A46" t="s">
         <v>52</v>
       </c>
@@ -2098,7 +2098,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:8">
+    <row r="47" spans="1:7">
       <c r="A47" t="s">
         <v>53</v>
       </c>
@@ -2106,7 +2106,7 @@
         <v>2551</v>
       </c>
       <c r="C47">
-        <v>615</v>
+        <v>549</v>
       </c>
       <c r="D47">
         <v>0</v>
@@ -2115,16 +2115,13 @@
         <v>0</v>
       </c>
       <c r="F47">
-        <v>3166</v>
+        <v>3100</v>
       </c>
       <c r="G47" t="b">
-        <v>0</v>
-      </c>
-      <c r="H47" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
       <c r="A48" t="s">
         <v>54</v>
       </c>
@@ -2135,10 +2132,10 @@
         <v>0</v>
       </c>
       <c r="D48">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E48">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F48">
         <v>2527</v>
@@ -2152,10 +2149,10 @@
         <v>55</v>
       </c>
       <c r="B49">
-        <v>2542</v>
+        <v>2543</v>
       </c>
       <c r="C49">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="D49">
         <v>0</v>
@@ -2164,7 +2161,7 @@
         <v>13</v>
       </c>
       <c r="F49">
-        <v>2542</v>
+        <v>2572</v>
       </c>
       <c r="G49" t="b">
         <v>1</v>
@@ -2175,7 +2172,7 @@
         <v>56</v>
       </c>
       <c r="B50">
-        <v>2549</v>
+        <v>2550</v>
       </c>
       <c r="C50">
         <v>0</v>
@@ -2184,7 +2181,7 @@
         <v>0</v>
       </c>
       <c r="E50">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F50">
         <v>2528</v>
@@ -2198,7 +2195,7 @@
         <v>57</v>
       </c>
       <c r="B51">
-        <v>2542</v>
+        <v>2543</v>
       </c>
       <c r="C51">
         <v>1</v>
@@ -2207,7 +2204,7 @@
         <v>2</v>
       </c>
       <c r="E51">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F51">
         <v>2528</v>
@@ -2267,7 +2264,7 @@
         <v>60</v>
       </c>
       <c r="B54">
-        <v>2001</v>
+        <v>2005</v>
       </c>
       <c r="C54">
         <v>0</v>
@@ -2276,7 +2273,7 @@
         <v>0</v>
       </c>
       <c r="E54">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="F54">
         <v>1840</v>
@@ -2290,7 +2287,7 @@
         <v>61</v>
       </c>
       <c r="B55">
-        <v>2573</v>
+        <v>2577</v>
       </c>
       <c r="C55">
         <v>0</v>
@@ -2299,7 +2296,7 @@
         <v>0</v>
       </c>
       <c r="E55">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F55">
         <v>2528</v>
@@ -2313,7 +2310,7 @@
         <v>62</v>
       </c>
       <c r="B56">
-        <v>2668</v>
+        <v>2674</v>
       </c>
       <c r="C56">
         <v>1</v>
@@ -2322,7 +2319,7 @@
         <v>0</v>
       </c>
       <c r="E56">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F56">
         <v>2529</v>
@@ -2336,7 +2333,7 @@
         <v>63</v>
       </c>
       <c r="B57">
-        <v>2739</v>
+        <v>2757</v>
       </c>
       <c r="C57">
         <v>4</v>
@@ -2345,10 +2342,10 @@
         <v>0</v>
       </c>
       <c r="E57">
-        <v>205</v>
+        <v>226</v>
       </c>
       <c r="F57">
-        <v>2538</v>
+        <v>2535</v>
       </c>
       <c r="G57" t="b">
         <v>1</v>
@@ -2359,7 +2356,7 @@
         <v>64</v>
       </c>
       <c r="B58">
-        <v>1909</v>
+        <v>1910</v>
       </c>
       <c r="C58">
         <v>1</v>
@@ -2368,7 +2365,7 @@
         <v>0</v>
       </c>
       <c r="E58">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F58">
         <v>1836</v>
@@ -2382,7 +2379,7 @@
         <v>65</v>
       </c>
       <c r="B59">
-        <v>2563</v>
+        <v>2564</v>
       </c>
       <c r="C59">
         <v>0</v>
@@ -2391,7 +2388,7 @@
         <v>0</v>
       </c>
       <c r="E59">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F59">
         <v>2528</v>
@@ -2405,7 +2402,7 @@
         <v>66</v>
       </c>
       <c r="B60">
-        <v>1891</v>
+        <v>1892</v>
       </c>
       <c r="C60">
         <v>0</v>
@@ -2414,7 +2411,7 @@
         <v>0</v>
       </c>
       <c r="E60">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F60">
         <v>1832</v>
@@ -2428,7 +2425,7 @@
         <v>67</v>
       </c>
       <c r="B61">
-        <v>1855</v>
+        <v>1856</v>
       </c>
       <c r="C61">
         <v>0</v>
@@ -2437,7 +2434,7 @@
         <v>2</v>
       </c>
       <c r="E61">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F61">
         <v>1827</v>
@@ -2451,7 +2448,7 @@
         <v>68</v>
       </c>
       <c r="B62">
-        <v>2616</v>
+        <v>2621</v>
       </c>
       <c r="C62">
         <v>0</v>
@@ -2460,7 +2457,7 @@
         <v>0</v>
       </c>
       <c r="E62">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="F62">
         <v>2532</v>
@@ -2474,7 +2471,7 @@
         <v>69</v>
       </c>
       <c r="B63">
-        <v>2615</v>
+        <v>2620</v>
       </c>
       <c r="C63">
         <v>1</v>
@@ -2483,7 +2480,7 @@
         <v>1</v>
       </c>
       <c r="E63">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F63">
         <v>2532</v>
@@ -2497,7 +2494,7 @@
         <v>70</v>
       </c>
       <c r="B64">
-        <v>2624</v>
+        <v>2629</v>
       </c>
       <c r="C64">
         <v>0</v>
@@ -2506,7 +2503,7 @@
         <v>1</v>
       </c>
       <c r="E64">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="F64">
         <v>2533</v>
@@ -2520,7 +2517,7 @@
         <v>71</v>
       </c>
       <c r="B65">
-        <v>2616</v>
+        <v>2621</v>
       </c>
       <c r="C65">
         <v>0</v>
@@ -2529,7 +2526,7 @@
         <v>0</v>
       </c>
       <c r="E65">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F65">
         <v>2531</v>
@@ -2543,7 +2540,7 @@
         <v>72</v>
       </c>
       <c r="B66">
-        <v>2622</v>
+        <v>2628</v>
       </c>
       <c r="C66">
         <v>2</v>
@@ -2552,7 +2549,7 @@
         <v>3</v>
       </c>
       <c r="E66">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="F66">
         <v>2532</v>
@@ -2566,7 +2563,7 @@
         <v>73</v>
       </c>
       <c r="B67">
-        <v>2614</v>
+        <v>2619</v>
       </c>
       <c r="C67">
         <v>1</v>
@@ -2575,7 +2572,7 @@
         <v>0</v>
       </c>
       <c r="E67">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="F67">
         <v>2532</v>
@@ -2589,7 +2586,7 @@
         <v>74</v>
       </c>
       <c r="B68">
-        <v>2619</v>
+        <v>2624</v>
       </c>
       <c r="C68">
         <v>0</v>
@@ -2598,7 +2595,7 @@
         <v>0</v>
       </c>
       <c r="E68">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="F68">
         <v>2531</v>
@@ -2612,7 +2609,7 @@
         <v>75</v>
       </c>
       <c r="B69">
-        <v>2619</v>
+        <v>2624</v>
       </c>
       <c r="C69">
         <v>0</v>
@@ -2621,7 +2618,7 @@
         <v>0</v>
       </c>
       <c r="E69">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="F69">
         <v>2532</v>
@@ -2635,7 +2632,7 @@
         <v>76</v>
       </c>
       <c r="B70">
-        <v>2623</v>
+        <v>2628</v>
       </c>
       <c r="C70">
         <v>1</v>
@@ -2644,7 +2641,7 @@
         <v>1</v>
       </c>
       <c r="E70">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="F70">
         <v>2532</v>
@@ -2658,7 +2655,7 @@
         <v>77</v>
       </c>
       <c r="B71">
-        <v>2617</v>
+        <v>2622</v>
       </c>
       <c r="C71">
         <v>0</v>
@@ -2667,7 +2664,7 @@
         <v>0</v>
       </c>
       <c r="E71">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F71">
         <v>2532</v>
@@ -2681,7 +2678,7 @@
         <v>78</v>
       </c>
       <c r="B72">
-        <v>2619</v>
+        <v>2624</v>
       </c>
       <c r="C72">
         <v>3</v>
@@ -2690,7 +2687,7 @@
         <v>1</v>
       </c>
       <c r="E72">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="F72">
         <v>2531</v>
@@ -2704,7 +2701,7 @@
         <v>79</v>
       </c>
       <c r="B73">
-        <v>2737</v>
+        <v>2751</v>
       </c>
       <c r="C73">
         <v>6</v>
@@ -2713,7 +2710,7 @@
         <v>0</v>
       </c>
       <c r="E73">
-        <v>184</v>
+        <v>198</v>
       </c>
       <c r="F73">
         <v>2559</v>
@@ -2727,7 +2724,7 @@
         <v>80</v>
       </c>
       <c r="B74">
-        <v>2609</v>
+        <v>2610</v>
       </c>
       <c r="C74">
         <v>0</v>
@@ -2736,7 +2733,7 @@
         <v>1</v>
       </c>
       <c r="E74">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F74">
         <v>2540</v>
@@ -2750,7 +2747,7 @@
         <v>81</v>
       </c>
       <c r="B75">
-        <v>2818</v>
+        <v>2847</v>
       </c>
       <c r="C75">
         <v>6</v>
@@ -2759,10 +2756,10 @@
         <v>1</v>
       </c>
       <c r="E75">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="F75">
-        <v>2615</v>
+        <v>2637</v>
       </c>
       <c r="G75" t="b">
         <v>1</v>
@@ -2773,7 +2770,7 @@
         <v>82</v>
       </c>
       <c r="B76">
-        <v>2834</v>
+        <v>2864</v>
       </c>
       <c r="C76">
         <v>12</v>
@@ -2785,7 +2782,7 @@
         <v>195</v>
       </c>
       <c r="F76">
-        <v>2653</v>
+        <v>2683</v>
       </c>
       <c r="G76" t="b">
         <v>1</v>
@@ -2796,7 +2793,7 @@
         <v>83</v>
       </c>
       <c r="B77">
-        <v>2828</v>
+        <v>2855</v>
       </c>
       <c r="C77">
         <v>5</v>
@@ -2805,10 +2802,10 @@
         <v>0</v>
       </c>
       <c r="E77">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="F77">
-        <v>2634</v>
+        <v>2654</v>
       </c>
       <c r="G77" t="b">
         <v>1</v>
@@ -2819,7 +2816,7 @@
         <v>84</v>
       </c>
       <c r="B78">
-        <v>2732</v>
+        <v>2747</v>
       </c>
       <c r="C78">
         <v>0</v>
@@ -2828,7 +2825,7 @@
         <v>1</v>
       </c>
       <c r="E78">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="F78">
         <v>2558</v>
@@ -2842,7 +2839,7 @@
         <v>85</v>
       </c>
       <c r="B79">
-        <v>2817</v>
+        <v>2844</v>
       </c>
       <c r="C79">
         <v>0</v>
@@ -2851,10 +2848,10 @@
         <v>1</v>
       </c>
       <c r="E79">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="F79">
-        <v>2632</v>
+        <v>2652</v>
       </c>
       <c r="G79" t="b">
         <v>1</v>
@@ -2865,7 +2862,7 @@
         <v>86</v>
       </c>
       <c r="B80">
-        <v>2604</v>
+        <v>2605</v>
       </c>
       <c r="C80">
         <v>0</v>
@@ -2874,7 +2871,7 @@
         <v>1</v>
       </c>
       <c r="E80">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F80">
         <v>2540</v>
@@ -2888,7 +2885,7 @@
         <v>87</v>
       </c>
       <c r="B81">
-        <v>2817</v>
+        <v>2846</v>
       </c>
       <c r="C81">
         <v>1</v>
@@ -2897,10 +2894,10 @@
         <v>0</v>
       </c>
       <c r="E81">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="F81">
-        <v>2613</v>
+        <v>2635</v>
       </c>
       <c r="G81" t="b">
         <v>1</v>
@@ -2911,7 +2908,7 @@
         <v>88</v>
       </c>
       <c r="B82">
-        <v>2838</v>
+        <v>2867</v>
       </c>
       <c r="C82">
         <v>3</v>
@@ -2920,10 +2917,10 @@
         <v>1</v>
       </c>
       <c r="E82">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="F82">
-        <v>2611</v>
+        <v>2633</v>
       </c>
       <c r="G82" t="b">
         <v>1</v>
@@ -2934,7 +2931,7 @@
         <v>89</v>
       </c>
       <c r="B83">
-        <v>2565</v>
+        <v>2572</v>
       </c>
       <c r="C83">
         <v>1</v>
@@ -2943,7 +2940,7 @@
         <v>0</v>
       </c>
       <c r="E83">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="F83">
         <v>2528</v>
@@ -2957,7 +2954,7 @@
         <v>90</v>
       </c>
       <c r="B84">
-        <v>2570</v>
+        <v>2577</v>
       </c>
       <c r="C84">
         <v>0</v>
@@ -2966,7 +2963,7 @@
         <v>0</v>
       </c>
       <c r="E84">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="F84">
         <v>2528</v>
@@ -2980,7 +2977,7 @@
         <v>91</v>
       </c>
       <c r="B85">
-        <v>2562</v>
+        <v>2568</v>
       </c>
       <c r="C85">
         <v>7</v>
@@ -2989,7 +2986,7 @@
         <v>0</v>
       </c>
       <c r="E85">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="F85">
         <v>2528</v>
@@ -3003,7 +3000,7 @@
         <v>92</v>
       </c>
       <c r="B86">
-        <v>2566</v>
+        <v>2573</v>
       </c>
       <c r="C86">
         <v>1</v>
@@ -3012,7 +3009,7 @@
         <v>0</v>
       </c>
       <c r="E86">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="F86">
         <v>2528</v>
@@ -3026,7 +3023,7 @@
         <v>93</v>
       </c>
       <c r="B87">
-        <v>2566</v>
+        <v>2572</v>
       </c>
       <c r="C87">
         <v>0</v>
@@ -3035,7 +3032,7 @@
         <v>1</v>
       </c>
       <c r="E87">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="F87">
         <v>2528</v>
@@ -3049,7 +3046,7 @@
         <v>94</v>
       </c>
       <c r="B88">
-        <v>2573</v>
+        <v>2582</v>
       </c>
       <c r="C88">
         <v>0</v>
@@ -3058,7 +3055,7 @@
         <v>1</v>
       </c>
       <c r="E88">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="F88">
         <v>2528</v>
@@ -3072,7 +3069,7 @@
         <v>95</v>
       </c>
       <c r="B89">
-        <v>2566</v>
+        <v>2573</v>
       </c>
       <c r="C89">
         <v>5</v>
@@ -3081,7 +3078,7 @@
         <v>0</v>
       </c>
       <c r="E89">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="F89">
         <v>2528</v>
@@ -3095,7 +3092,7 @@
         <v>96</v>
       </c>
       <c r="B90">
-        <v>2564</v>
+        <v>2570</v>
       </c>
       <c r="C90">
         <v>0</v>
@@ -3104,7 +3101,7 @@
         <v>0</v>
       </c>
       <c r="E90">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="F90">
         <v>2528</v>
@@ -3118,7 +3115,7 @@
         <v>97</v>
       </c>
       <c r="B91">
-        <v>2566</v>
+        <v>2573</v>
       </c>
       <c r="C91">
         <v>0</v>
@@ -3127,7 +3124,7 @@
         <v>0</v>
       </c>
       <c r="E91">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="F91">
         <v>2528</v>
@@ -3141,7 +3138,7 @@
         <v>98</v>
       </c>
       <c r="B92">
-        <v>2582</v>
+        <v>2583</v>
       </c>
       <c r="C92">
         <v>1</v>
@@ -3150,7 +3147,7 @@
         <v>0</v>
       </c>
       <c r="E92">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F92">
         <v>2528</v>
@@ -3164,7 +3161,7 @@
         <v>99</v>
       </c>
       <c r="B93">
-        <v>2585</v>
+        <v>2586</v>
       </c>
       <c r="C93">
         <v>0</v>
@@ -3173,7 +3170,7 @@
         <v>0</v>
       </c>
       <c r="E93">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F93">
         <v>2528</v>
@@ -3187,7 +3184,7 @@
         <v>100</v>
       </c>
       <c r="B94">
-        <v>2584</v>
+        <v>2585</v>
       </c>
       <c r="C94">
         <v>8</v>
@@ -3196,7 +3193,7 @@
         <v>0</v>
       </c>
       <c r="E94">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F94">
         <v>2528</v>
@@ -3210,7 +3207,7 @@
         <v>101</v>
       </c>
       <c r="B95">
-        <v>2579</v>
+        <v>2580</v>
       </c>
       <c r="C95">
         <v>5</v>
@@ -3219,7 +3216,7 @@
         <v>0</v>
       </c>
       <c r="E95">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F95">
         <v>2528</v>
@@ -3233,7 +3230,7 @@
         <v>102</v>
       </c>
       <c r="B96">
-        <v>2581</v>
+        <v>2582</v>
       </c>
       <c r="C96">
         <v>1</v>
@@ -3242,7 +3239,7 @@
         <v>0</v>
       </c>
       <c r="E96">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F96">
         <v>2528</v>
@@ -3256,7 +3253,7 @@
         <v>103</v>
       </c>
       <c r="B97">
-        <v>2583</v>
+        <v>2584</v>
       </c>
       <c r="C97">
         <v>7</v>
@@ -3265,7 +3262,7 @@
         <v>18</v>
       </c>
       <c r="E97">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F97">
         <v>2528</v>
@@ -3279,7 +3276,7 @@
         <v>104</v>
       </c>
       <c r="B98">
-        <v>2581</v>
+        <v>2582</v>
       </c>
       <c r="C98">
         <v>15</v>
@@ -3288,7 +3285,7 @@
         <v>0</v>
       </c>
       <c r="E98">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F98">
         <v>2528</v>
@@ -3302,7 +3299,7 @@
         <v>105</v>
       </c>
       <c r="B99">
-        <v>2583</v>
+        <v>2584</v>
       </c>
       <c r="C99">
         <v>1</v>
@@ -3311,7 +3308,7 @@
         <v>3</v>
       </c>
       <c r="E99">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F99">
         <v>2529</v>
@@ -3325,7 +3322,7 @@
         <v>106</v>
       </c>
       <c r="B100">
-        <v>2584</v>
+        <v>2585</v>
       </c>
       <c r="C100">
         <v>0</v>
@@ -3334,7 +3331,7 @@
         <v>0</v>
       </c>
       <c r="E100">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F100">
         <v>2528</v>
@@ -3348,7 +3345,7 @@
         <v>107</v>
       </c>
       <c r="B101">
-        <v>2588</v>
+        <v>2592</v>
       </c>
       <c r="C101">
         <v>3</v>
@@ -3357,7 +3354,7 @@
         <v>0</v>
       </c>
       <c r="E101">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="F101">
         <v>2528</v>
@@ -3371,7 +3368,7 @@
         <v>108</v>
       </c>
       <c r="B102">
-        <v>2587</v>
+        <v>2589</v>
       </c>
       <c r="C102">
         <v>1</v>
@@ -3380,7 +3377,7 @@
         <v>0</v>
       </c>
       <c r="E102">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F102">
         <v>2528</v>
@@ -3394,7 +3391,7 @@
         <v>109</v>
       </c>
       <c r="B103">
-        <v>2588</v>
+        <v>2589</v>
       </c>
       <c r="C103">
         <v>0</v>
@@ -3403,7 +3400,7 @@
         <v>1</v>
       </c>
       <c r="E103">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F103">
         <v>2528</v>
@@ -3417,7 +3414,7 @@
         <v>110</v>
       </c>
       <c r="B104">
-        <v>2620</v>
+        <v>2626</v>
       </c>
       <c r="C104">
         <v>1</v>
@@ -3426,7 +3423,7 @@
         <v>2</v>
       </c>
       <c r="E104">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F104">
         <v>2542</v>
@@ -3440,7 +3437,7 @@
         <v>111</v>
       </c>
       <c r="B105">
-        <v>2616</v>
+        <v>2623</v>
       </c>
       <c r="C105">
         <v>0</v>
@@ -3449,7 +3446,7 @@
         <v>4</v>
       </c>
       <c r="E105">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="F105">
         <v>2542</v>
@@ -3463,7 +3460,7 @@
         <v>112</v>
       </c>
       <c r="B106">
-        <v>2613</v>
+        <v>2620</v>
       </c>
       <c r="C106">
         <v>0</v>
@@ -3472,7 +3469,7 @@
         <v>4</v>
       </c>
       <c r="E106">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="F106">
         <v>2542</v>
@@ -3486,7 +3483,7 @@
         <v>113</v>
       </c>
       <c r="B107">
-        <v>2616</v>
+        <v>2623</v>
       </c>
       <c r="C107">
         <v>1</v>
@@ -3495,7 +3492,7 @@
         <v>22</v>
       </c>
       <c r="E107">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="F107">
         <v>2542</v>
@@ -3509,7 +3506,7 @@
         <v>114</v>
       </c>
       <c r="B108">
-        <v>2613</v>
+        <v>2618</v>
       </c>
       <c r="C108">
         <v>0</v>
@@ -3518,7 +3515,7 @@
         <v>0</v>
       </c>
       <c r="E108">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="F108">
         <v>2542</v>
@@ -3532,7 +3529,7 @@
         <v>115</v>
       </c>
       <c r="B109">
-        <v>2615</v>
+        <v>2622</v>
       </c>
       <c r="C109">
         <v>0</v>
@@ -3541,7 +3538,7 @@
         <v>27</v>
       </c>
       <c r="E109">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="F109">
         <v>2542</v>
@@ -3555,7 +3552,7 @@
         <v>116</v>
       </c>
       <c r="B110">
-        <v>2614</v>
+        <v>2621</v>
       </c>
       <c r="C110">
         <v>4</v>
@@ -3564,7 +3561,7 @@
         <v>1</v>
       </c>
       <c r="E110">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="F110">
         <v>2542</v>
@@ -3578,7 +3575,7 @@
         <v>117</v>
       </c>
       <c r="B111">
-        <v>2617</v>
+        <v>2624</v>
       </c>
       <c r="C111">
         <v>0</v>
@@ -3587,7 +3584,7 @@
         <v>4</v>
       </c>
       <c r="E111">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="F111">
         <v>2542</v>
@@ -3601,7 +3598,7 @@
         <v>118</v>
       </c>
       <c r="B112">
-        <v>2612</v>
+        <v>2619</v>
       </c>
       <c r="C112">
         <v>3</v>
@@ -3610,7 +3607,7 @@
         <v>0</v>
       </c>
       <c r="E112">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="F112">
         <v>2542</v>
@@ -3624,7 +3621,7 @@
         <v>119</v>
       </c>
       <c r="B113">
-        <v>2594</v>
+        <v>2604</v>
       </c>
       <c r="C113">
         <v>0</v>
@@ -3633,10 +3630,10 @@
         <v>2</v>
       </c>
       <c r="E113">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="F113">
-        <v>2529</v>
+        <v>2530</v>
       </c>
       <c r="G113" t="b">
         <v>1</v>
@@ -3647,7 +3644,7 @@
         <v>120</v>
       </c>
       <c r="B114">
-        <v>2637</v>
+        <v>2645</v>
       </c>
       <c r="C114">
         <v>1</v>
@@ -3656,7 +3653,7 @@
         <v>0</v>
       </c>
       <c r="E114">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="F114">
         <v>2535</v>
@@ -3670,7 +3667,7 @@
         <v>121</v>
       </c>
       <c r="B115">
-        <v>2626</v>
+        <v>2634</v>
       </c>
       <c r="C115">
         <v>0</v>
@@ -3679,7 +3676,7 @@
         <v>0</v>
       </c>
       <c r="E115">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="F115">
         <v>2529</v>
@@ -3739,7 +3736,7 @@
         <v>124</v>
       </c>
       <c r="B118">
-        <v>2563</v>
+        <v>2564</v>
       </c>
       <c r="C118">
         <v>0</v>
@@ -3748,7 +3745,7 @@
         <v>0</v>
       </c>
       <c r="E118">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F118">
         <v>2533</v>
@@ -3877,7 +3874,7 @@
         <v>130</v>
       </c>
       <c r="B124">
-        <v>2632</v>
+        <v>2641</v>
       </c>
       <c r="C124">
         <v>1</v>
@@ -3886,7 +3883,7 @@
         <v>0</v>
       </c>
       <c r="E124">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="F124">
         <v>2529</v>
@@ -3946,7 +3943,7 @@
         <v>133</v>
       </c>
       <c r="B127">
-        <v>2614</v>
+        <v>2621</v>
       </c>
       <c r="C127">
         <v>0</v>
@@ -3955,10 +3952,10 @@
         <v>0</v>
       </c>
       <c r="E127">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="F127">
-        <v>2533</v>
+        <v>2532</v>
       </c>
       <c r="G127" t="b">
         <v>1</v>
@@ -3992,7 +3989,7 @@
         <v>135</v>
       </c>
       <c r="B129">
-        <v>2608</v>
+        <v>2615</v>
       </c>
       <c r="C129">
         <v>0</v>
@@ -4001,10 +3998,10 @@
         <v>0</v>
       </c>
       <c r="E129">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="F129">
-        <v>2530</v>
+        <v>2529</v>
       </c>
       <c r="G129" t="b">
         <v>1</v>
@@ -4015,7 +4012,7 @@
         <v>136</v>
       </c>
       <c r="B130">
-        <v>2625</v>
+        <v>2635</v>
       </c>
       <c r="C130">
         <v>0</v>
@@ -4024,7 +4021,7 @@
         <v>0</v>
       </c>
       <c r="E130">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="F130">
         <v>2525</v>
@@ -4038,7 +4035,7 @@
         <v>137</v>
       </c>
       <c r="B131">
-        <v>2626</v>
+        <v>2635</v>
       </c>
       <c r="C131">
         <v>1</v>
@@ -4047,7 +4044,7 @@
         <v>0</v>
       </c>
       <c r="E131">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="F131">
         <v>2529</v>
@@ -4061,7 +4058,7 @@
         <v>138</v>
       </c>
       <c r="B132">
-        <v>2611</v>
+        <v>2618</v>
       </c>
       <c r="C132">
         <v>0</v>
@@ -4070,10 +4067,10 @@
         <v>0</v>
       </c>
       <c r="E132">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="F132">
-        <v>2533</v>
+        <v>2532</v>
       </c>
       <c r="G132" t="b">
         <v>1</v>
@@ -4107,7 +4104,7 @@
         <v>140</v>
       </c>
       <c r="B134">
-        <v>2628</v>
+        <v>2637</v>
       </c>
       <c r="C134">
         <v>0</v>
@@ -4116,7 +4113,7 @@
         <v>1</v>
       </c>
       <c r="E134">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="F134">
         <v>2529</v>
@@ -4130,7 +4127,7 @@
         <v>141</v>
       </c>
       <c r="B135">
-        <v>2627</v>
+        <v>2629</v>
       </c>
       <c r="C135">
         <v>0</v>
@@ -4139,7 +4136,7 @@
         <v>0</v>
       </c>
       <c r="E135">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F135">
         <v>2544</v>
@@ -4153,7 +4150,7 @@
         <v>142</v>
       </c>
       <c r="B136">
-        <v>2630</v>
+        <v>2643</v>
       </c>
       <c r="C136">
         <v>0</v>
@@ -4162,10 +4159,10 @@
         <v>0</v>
       </c>
       <c r="E136">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="F136">
-        <v>2527</v>
+        <v>2526</v>
       </c>
       <c r="G136" t="b">
         <v>1</v>
@@ -4176,7 +4173,7 @@
         <v>143</v>
       </c>
       <c r="B137">
-        <v>2557</v>
+        <v>2559</v>
       </c>
       <c r="C137">
         <v>1</v>
@@ -4185,7 +4182,7 @@
         <v>0</v>
       </c>
       <c r="E137">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F137">
         <v>2529</v>
@@ -4199,7 +4196,7 @@
         <v>144</v>
       </c>
       <c r="B138">
-        <v>2555</v>
+        <v>2558</v>
       </c>
       <c r="C138">
         <v>0</v>
@@ -4208,7 +4205,7 @@
         <v>0</v>
       </c>
       <c r="E138">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F138">
         <v>2529</v>
@@ -4222,7 +4219,7 @@
         <v>145</v>
       </c>
       <c r="B139">
-        <v>2543</v>
+        <v>2544</v>
       </c>
       <c r="C139">
         <v>0</v>
@@ -4231,10 +4228,10 @@
         <v>0</v>
       </c>
       <c r="E139">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F139">
-        <v>2526</v>
+        <v>2525</v>
       </c>
       <c r="G139" t="b">
         <v>1</v>
@@ -4245,7 +4242,7 @@
         <v>146</v>
       </c>
       <c r="B140">
-        <v>2551</v>
+        <v>2554</v>
       </c>
       <c r="C140">
         <v>0</v>
@@ -4254,7 +4251,7 @@
         <v>0</v>
       </c>
       <c r="E140">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F140">
         <v>2527</v>
@@ -4268,7 +4265,7 @@
         <v>147</v>
       </c>
       <c r="B141">
-        <v>2703</v>
+        <v>2720</v>
       </c>
       <c r="C141">
         <v>0</v>
@@ -4277,10 +4274,10 @@
         <v>0</v>
       </c>
       <c r="E141">
-        <v>169</v>
+        <v>188</v>
       </c>
       <c r="F141">
-        <v>2534</v>
+        <v>2532</v>
       </c>
       <c r="G141" t="b">
         <v>1</v>
@@ -4291,7 +4288,7 @@
         <v>148</v>
       </c>
       <c r="B142">
-        <v>2681</v>
+        <v>2689</v>
       </c>
       <c r="C142">
         <v>0</v>
@@ -4300,7 +4297,7 @@
         <v>0</v>
       </c>
       <c r="E142">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="F142">
         <v>2527</v>
@@ -4337,7 +4334,7 @@
         <v>150</v>
       </c>
       <c r="B144">
-        <v>2701</v>
+        <v>2703</v>
       </c>
       <c r="C144">
         <v>0</v>
@@ -4346,7 +4343,7 @@
         <v>0</v>
       </c>
       <c r="E144">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F144">
         <v>2527</v>
@@ -4360,7 +4357,7 @@
         <v>151</v>
       </c>
       <c r="B145">
-        <v>2931</v>
+        <v>2948</v>
       </c>
       <c r="C145">
         <v>0</v>
@@ -4369,10 +4366,10 @@
         <v>0</v>
       </c>
       <c r="E145">
-        <v>256</v>
+        <v>272</v>
       </c>
       <c r="F145">
-        <v>2675</v>
+        <v>2676</v>
       </c>
       <c r="G145" t="b">
         <v>1</v>
@@ -4383,7 +4380,7 @@
         <v>152</v>
       </c>
       <c r="B146">
-        <v>2552</v>
+        <v>2553</v>
       </c>
       <c r="C146">
         <v>0</v>
@@ -4392,7 +4389,7 @@
         <v>0</v>
       </c>
       <c r="E146">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F146">
         <v>2529</v>
@@ -4406,7 +4403,7 @@
         <v>153</v>
       </c>
       <c r="B147">
-        <v>2565</v>
+        <v>2566</v>
       </c>
       <c r="C147">
         <v>0</v>
@@ -4418,7 +4415,7 @@
         <v>37</v>
       </c>
       <c r="F147">
-        <v>2528</v>
+        <v>2529</v>
       </c>
       <c r="G147" t="b">
         <v>1</v>
@@ -4429,7 +4426,7 @@
         <v>154</v>
       </c>
       <c r="B148">
-        <v>2823</v>
+        <v>2843</v>
       </c>
       <c r="C148">
         <v>1</v>
@@ -4438,10 +4435,10 @@
         <v>1</v>
       </c>
       <c r="E148">
-        <v>282</v>
+        <v>306</v>
       </c>
       <c r="F148">
-        <v>2543</v>
+        <v>2539</v>
       </c>
       <c r="G148" t="b">
         <v>1</v>
@@ -4452,7 +4449,7 @@
         <v>155</v>
       </c>
       <c r="B149">
-        <v>2951</v>
+        <v>2959</v>
       </c>
       <c r="C149">
         <v>0</v>
@@ -4461,7 +4458,7 @@
         <v>0</v>
       </c>
       <c r="E149">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="F149">
         <v>2765</v>
@@ -4475,7 +4472,7 @@
         <v>156</v>
       </c>
       <c r="B150">
-        <v>2754</v>
+        <v>2760</v>
       </c>
       <c r="C150">
         <v>0</v>
@@ -4484,7 +4481,7 @@
         <v>0</v>
       </c>
       <c r="E150">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="F150">
         <v>2528</v>
@@ -4498,7 +4495,7 @@
         <v>157</v>
       </c>
       <c r="B151">
-        <v>2550</v>
+        <v>2551</v>
       </c>
       <c r="C151">
         <v>0</v>
@@ -4507,7 +4504,7 @@
         <v>0</v>
       </c>
       <c r="E151">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F151">
         <v>2528</v>
@@ -4521,7 +4518,7 @@
         <v>158</v>
       </c>
       <c r="B152">
-        <v>1849</v>
+        <v>1850</v>
       </c>
       <c r="C152">
         <v>0</v>
@@ -4530,7 +4527,7 @@
         <v>0</v>
       </c>
       <c r="E152">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F152">
         <v>1830</v>
@@ -4544,7 +4541,7 @@
         <v>159</v>
       </c>
       <c r="B153">
-        <v>2544</v>
+        <v>2545</v>
       </c>
       <c r="C153">
         <v>0</v>
@@ -4553,7 +4550,7 @@
         <v>0</v>
       </c>
       <c r="E153">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F153">
         <v>2528</v>
@@ -4567,7 +4564,7 @@
         <v>160</v>
       </c>
       <c r="B154">
-        <v>2547</v>
+        <v>2548</v>
       </c>
       <c r="C154">
         <v>1</v>
@@ -4576,7 +4573,7 @@
         <v>0</v>
       </c>
       <c r="E154">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F154">
         <v>2528</v>
@@ -4590,7 +4587,7 @@
         <v>161</v>
       </c>
       <c r="B155">
-        <v>2546</v>
+        <v>2547</v>
       </c>
       <c r="C155">
         <v>0</v>
@@ -4599,7 +4596,7 @@
         <v>0</v>
       </c>
       <c r="E155">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F155">
         <v>2528</v>
@@ -4613,7 +4610,7 @@
         <v>162</v>
       </c>
       <c r="B156">
-        <v>2546</v>
+        <v>2547</v>
       </c>
       <c r="C156">
         <v>0</v>
@@ -4622,7 +4619,7 @@
         <v>0</v>
       </c>
       <c r="E156">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F156">
         <v>2528</v>
@@ -4636,7 +4633,7 @@
         <v>163</v>
       </c>
       <c r="B157">
-        <v>2548</v>
+        <v>2549</v>
       </c>
       <c r="C157">
         <v>0</v>
@@ -4645,7 +4642,7 @@
         <v>0</v>
       </c>
       <c r="E157">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F157">
         <v>2528</v>
@@ -4659,7 +4656,7 @@
         <v>164</v>
       </c>
       <c r="B158">
-        <v>2545</v>
+        <v>2546</v>
       </c>
       <c r="C158">
         <v>0</v>
@@ -4668,7 +4665,7 @@
         <v>0</v>
       </c>
       <c r="E158">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F158">
         <v>2528</v>
@@ -4682,7 +4679,7 @@
         <v>165</v>
       </c>
       <c r="B159">
-        <v>2545</v>
+        <v>2546</v>
       </c>
       <c r="C159">
         <v>0</v>
@@ -4691,7 +4688,7 @@
         <v>0</v>
       </c>
       <c r="E159">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F159">
         <v>2528</v>
@@ -4705,7 +4702,7 @@
         <v>166</v>
       </c>
       <c r="B160">
-        <v>2547</v>
+        <v>2548</v>
       </c>
       <c r="C160">
         <v>0</v>
@@ -4714,7 +4711,7 @@
         <v>0</v>
       </c>
       <c r="E160">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F160">
         <v>2528</v>
@@ -4728,7 +4725,7 @@
         <v>167</v>
       </c>
       <c r="B161">
-        <v>2547</v>
+        <v>2548</v>
       </c>
       <c r="C161">
         <v>0</v>
@@ -4737,7 +4734,7 @@
         <v>0</v>
       </c>
       <c r="E161">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F161">
         <v>2529</v>
@@ -4751,16 +4748,16 @@
         <v>168</v>
       </c>
       <c r="B162">
-        <v>2543</v>
+        <v>2544</v>
       </c>
       <c r="C162">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D162">
         <v>0</v>
       </c>
       <c r="E162">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F162">
         <v>2528</v>
@@ -4774,7 +4771,7 @@
         <v>169</v>
       </c>
       <c r="B163">
-        <v>2558</v>
+        <v>2560</v>
       </c>
       <c r="C163">
         <v>0</v>
@@ -4783,7 +4780,7 @@
         <v>1</v>
       </c>
       <c r="E163">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F163">
         <v>2528</v>
@@ -4820,7 +4817,7 @@
         <v>171</v>
       </c>
       <c r="B165">
-        <v>2553</v>
+        <v>2555</v>
       </c>
       <c r="C165">
         <v>1</v>
@@ -4829,7 +4826,7 @@
         <v>0</v>
       </c>
       <c r="E165">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F165">
         <v>2528</v>
@@ -4843,7 +4840,7 @@
         <v>172</v>
       </c>
       <c r="B166">
-        <v>1854</v>
+        <v>1856</v>
       </c>
       <c r="C166">
         <v>0</v>
@@ -4852,7 +4849,7 @@
         <v>0</v>
       </c>
       <c r="E166">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F166">
         <v>1830</v>
@@ -4866,7 +4863,7 @@
         <v>173</v>
       </c>
       <c r="B167">
-        <v>2547</v>
+        <v>2548</v>
       </c>
       <c r="C167">
         <v>0</v>
@@ -4875,7 +4872,7 @@
         <v>0</v>
       </c>
       <c r="E167">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F167">
         <v>2528</v>
@@ -4889,7 +4886,7 @@
         <v>174</v>
       </c>
       <c r="B168">
-        <v>2573</v>
+        <v>2574</v>
       </c>
       <c r="C168">
         <v>0</v>
@@ -4898,7 +4895,7 @@
         <v>3</v>
       </c>
       <c r="E168">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F168">
         <v>2528</v>
@@ -4935,7 +4932,7 @@
         <v>176</v>
       </c>
       <c r="B170">
-        <v>2547</v>
+        <v>2548</v>
       </c>
       <c r="C170">
         <v>0</v>
@@ -4944,7 +4941,7 @@
         <v>0</v>
       </c>
       <c r="E170">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F170">
         <v>2528</v>
@@ -4981,7 +4978,7 @@
         <v>178</v>
       </c>
       <c r="B172">
-        <v>2541</v>
+        <v>2542</v>
       </c>
       <c r="C172">
         <v>2</v>
@@ -4993,7 +4990,7 @@
         <v>17</v>
       </c>
       <c r="F172">
-        <v>2527</v>
+        <v>2528</v>
       </c>
       <c r="G172" t="b">
         <v>1</v>
@@ -5004,16 +5001,16 @@
         <v>179</v>
       </c>
       <c r="B173">
-        <v>2544</v>
+        <v>2545</v>
       </c>
       <c r="C173">
         <v>0</v>
       </c>
       <c r="D173">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E173">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F173">
         <v>2528</v>
@@ -5027,7 +5024,7 @@
         <v>180</v>
       </c>
       <c r="B174">
-        <v>2903</v>
+        <v>2928</v>
       </c>
       <c r="C174">
         <v>0</v>
@@ -5036,10 +5033,10 @@
         <v>0</v>
       </c>
       <c r="E174">
-        <v>318</v>
+        <v>337</v>
       </c>
       <c r="F174">
-        <v>2585</v>
+        <v>2591</v>
       </c>
       <c r="G174" t="b">
         <v>1</v>
@@ -5050,7 +5047,7 @@
         <v>181</v>
       </c>
       <c r="B175">
-        <v>2548</v>
+        <v>2549</v>
       </c>
       <c r="C175">
         <v>0</v>
@@ -5059,7 +5056,7 @@
         <v>0</v>
       </c>
       <c r="E175">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F175">
         <v>2528</v>
@@ -5073,7 +5070,7 @@
         <v>182</v>
       </c>
       <c r="B176">
-        <v>2549</v>
+        <v>2552</v>
       </c>
       <c r="C176">
         <v>0</v>
@@ -5082,7 +5079,7 @@
         <v>1</v>
       </c>
       <c r="E176">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F176">
         <v>2525</v>
@@ -5096,7 +5093,7 @@
         <v>183</v>
       </c>
       <c r="B177">
-        <v>2689</v>
+        <v>2719</v>
       </c>
       <c r="C177">
         <v>0</v>
@@ -5108,7 +5105,7 @@
         <v>35</v>
       </c>
       <c r="F177">
-        <v>2654</v>
+        <v>2684</v>
       </c>
       <c r="G177" t="b">
         <v>1</v>
@@ -5119,16 +5116,16 @@
         <v>184</v>
       </c>
       <c r="B178">
-        <v>2937</v>
+        <v>2946</v>
       </c>
       <c r="C178">
         <v>0</v>
       </c>
       <c r="D178">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E178">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="F178">
         <v>2751</v>
@@ -5142,7 +5139,7 @@
         <v>185</v>
       </c>
       <c r="B179">
-        <v>2933</v>
+        <v>2950</v>
       </c>
       <c r="C179">
         <v>0</v>
@@ -5151,10 +5148,10 @@
         <v>0</v>
       </c>
       <c r="E179">
-        <v>331</v>
+        <v>347</v>
       </c>
       <c r="F179">
-        <v>2602</v>
+        <v>2603</v>
       </c>
       <c r="G179" t="b">
         <v>1</v>
@@ -5165,7 +5162,7 @@
         <v>186</v>
       </c>
       <c r="B180">
-        <v>2915</v>
+        <v>2928</v>
       </c>
       <c r="C180">
         <v>1</v>
@@ -5174,10 +5171,10 @@
         <v>2</v>
       </c>
       <c r="E180">
-        <v>310</v>
+        <v>322</v>
       </c>
       <c r="F180">
-        <v>2608</v>
+        <v>2609</v>
       </c>
       <c r="G180" t="b">
         <v>1</v>
@@ -5188,7 +5185,7 @@
         <v>187</v>
       </c>
       <c r="B181">
-        <v>2925</v>
+        <v>2942</v>
       </c>
       <c r="C181">
         <v>0</v>
@@ -5197,10 +5194,10 @@
         <v>0</v>
       </c>
       <c r="E181">
-        <v>323</v>
+        <v>339</v>
       </c>
       <c r="F181">
-        <v>2602</v>
+        <v>2603</v>
       </c>
       <c r="G181" t="b">
         <v>1</v>
@@ -5211,7 +5208,7 @@
         <v>188</v>
       </c>
       <c r="B182">
-        <v>2930</v>
+        <v>2947</v>
       </c>
       <c r="C182">
         <v>0</v>
@@ -5220,10 +5217,10 @@
         <v>1</v>
       </c>
       <c r="E182">
-        <v>326</v>
+        <v>342</v>
       </c>
       <c r="F182">
-        <v>2605</v>
+        <v>2606</v>
       </c>
       <c r="G182" t="b">
         <v>1</v>
@@ -5234,7 +5231,7 @@
         <v>189</v>
       </c>
       <c r="B183">
-        <v>2943</v>
+        <v>2962</v>
       </c>
       <c r="C183">
         <v>0</v>
@@ -5243,7 +5240,7 @@
         <v>0</v>
       </c>
       <c r="E183">
-        <v>341</v>
+        <v>360</v>
       </c>
       <c r="F183">
         <v>2602</v>
@@ -5257,7 +5254,7 @@
         <v>190</v>
       </c>
       <c r="B184">
-        <v>2910</v>
+        <v>2927</v>
       </c>
       <c r="C184">
         <v>0</v>
@@ -5266,10 +5263,10 @@
         <v>0</v>
       </c>
       <c r="E184">
-        <v>344</v>
+        <v>360</v>
       </c>
       <c r="F184">
-        <v>2566</v>
+        <v>2567</v>
       </c>
       <c r="G184" t="b">
         <v>1</v>
@@ -5303,7 +5300,7 @@
         <v>192</v>
       </c>
       <c r="B186">
-        <v>2543</v>
+        <v>2544</v>
       </c>
       <c r="C186">
         <v>0</v>
@@ -5312,7 +5309,7 @@
         <v>1</v>
       </c>
       <c r="E186">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F186">
         <v>2529</v>
@@ -5326,7 +5323,7 @@
         <v>193</v>
       </c>
       <c r="B187">
-        <v>2590</v>
+        <v>2593</v>
       </c>
       <c r="C187">
         <v>0</v>
@@ -5335,7 +5332,7 @@
         <v>0</v>
       </c>
       <c r="E187">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F187">
         <v>2530</v>
@@ -5349,7 +5346,7 @@
         <v>194</v>
       </c>
       <c r="B188">
-        <v>2547</v>
+        <v>2548</v>
       </c>
       <c r="C188">
         <v>0</v>
@@ -5358,7 +5355,7 @@
         <v>0</v>
       </c>
       <c r="E188">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F188">
         <v>2528</v>
@@ -5372,7 +5369,7 @@
         <v>195</v>
       </c>
       <c r="B189">
-        <v>2588</v>
+        <v>2589</v>
       </c>
       <c r="C189">
         <v>0</v>
@@ -5381,7 +5378,7 @@
         <v>0</v>
       </c>
       <c r="E189">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F189">
         <v>2531</v>
@@ -5487,7 +5484,7 @@
         <v>200</v>
       </c>
       <c r="B194">
-        <v>2618</v>
+        <v>2625</v>
       </c>
       <c r="C194">
         <v>1</v>
@@ -5496,10 +5493,10 @@
         <v>0</v>
       </c>
       <c r="E194">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="F194">
-        <v>2539</v>
+        <v>2541</v>
       </c>
       <c r="G194" t="b">
         <v>1</v>
@@ -5533,7 +5530,7 @@
         <v>202</v>
       </c>
       <c r="B196">
-        <v>2741</v>
+        <v>2746</v>
       </c>
       <c r="C196">
         <v>0</v>
@@ -5542,10 +5539,10 @@
         <v>13</v>
       </c>
       <c r="E196">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="F196">
-        <v>2634</v>
+        <v>2633</v>
       </c>
       <c r="G196" t="b">
         <v>1</v>
@@ -5556,7 +5553,7 @@
         <v>203</v>
       </c>
       <c r="B197">
-        <v>1873</v>
+        <v>1880</v>
       </c>
       <c r="C197">
         <v>0</v>
@@ -5565,7 +5562,7 @@
         <v>0</v>
       </c>
       <c r="E197">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="F197">
         <v>1831</v>
@@ -5579,7 +5576,7 @@
         <v>204</v>
       </c>
       <c r="B198">
-        <v>2743</v>
+        <v>2748</v>
       </c>
       <c r="C198">
         <v>2</v>
@@ -5588,10 +5585,10 @@
         <v>1</v>
       </c>
       <c r="E198">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="F198">
-        <v>2635</v>
+        <v>2634</v>
       </c>
       <c r="G198" t="b">
         <v>1</v>
@@ -5602,7 +5599,7 @@
         <v>205</v>
       </c>
       <c r="B199">
-        <v>2614</v>
+        <v>2621</v>
       </c>
       <c r="C199">
         <v>0</v>
@@ -5611,10 +5608,10 @@
         <v>0</v>
       </c>
       <c r="E199">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="F199">
-        <v>2533</v>
+        <v>2532</v>
       </c>
       <c r="G199" t="b">
         <v>1</v>
@@ -5625,7 +5622,7 @@
         <v>206</v>
       </c>
       <c r="B200">
-        <v>3165</v>
+        <v>3195</v>
       </c>
       <c r="C200">
         <v>0</v>
@@ -5637,7 +5634,7 @@
         <v>0</v>
       </c>
       <c r="F200">
-        <v>3165</v>
+        <v>3195</v>
       </c>
       <c r="G200" t="b">
         <v>1</v>
@@ -5648,7 +5645,7 @@
         <v>207</v>
       </c>
       <c r="B201">
-        <v>3165</v>
+        <v>3195</v>
       </c>
       <c r="C201">
         <v>1</v>
@@ -5660,7 +5657,7 @@
         <v>0</v>
       </c>
       <c r="F201">
-        <v>3166</v>
+        <v>3196</v>
       </c>
       <c r="G201" t="b">
         <v>0</v>
@@ -5674,7 +5671,7 @@
         <v>208</v>
       </c>
       <c r="B202">
-        <v>2869</v>
+        <v>2899</v>
       </c>
       <c r="C202">
         <v>0</v>
@@ -5686,7 +5683,7 @@
         <v>299</v>
       </c>
       <c r="F202">
-        <v>2570</v>
+        <v>2600</v>
       </c>
       <c r="G202" t="b">
         <v>1</v>
@@ -5697,7 +5694,7 @@
         <v>209</v>
       </c>
       <c r="B203">
-        <v>2544</v>
+        <v>2545</v>
       </c>
       <c r="C203">
         <v>0</v>
@@ -5706,7 +5703,7 @@
         <v>0</v>
       </c>
       <c r="E203">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F203">
         <v>2528</v>
@@ -5720,7 +5717,7 @@
         <v>210</v>
       </c>
       <c r="B204">
-        <v>2552</v>
+        <v>2553</v>
       </c>
       <c r="C204">
         <v>0</v>
@@ -5729,7 +5726,7 @@
         <v>0</v>
       </c>
       <c r="E204">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F204">
         <v>2526</v>
@@ -5743,7 +5740,7 @@
         <v>211</v>
       </c>
       <c r="B205">
-        <v>2543</v>
+        <v>2544</v>
       </c>
       <c r="C205">
         <v>0</v>
@@ -5752,7 +5749,7 @@
         <v>0</v>
       </c>
       <c r="E205">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F205">
         <v>2529</v>
@@ -5789,7 +5786,7 @@
         <v>213</v>
       </c>
       <c r="B207">
-        <v>2544</v>
+        <v>2545</v>
       </c>
       <c r="C207">
         <v>0</v>
@@ -5798,7 +5795,7 @@
         <v>0</v>
       </c>
       <c r="E207">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F207">
         <v>2529</v>
@@ -5858,7 +5855,7 @@
         <v>216</v>
       </c>
       <c r="B210">
-        <v>2542</v>
+        <v>2543</v>
       </c>
       <c r="C210">
         <v>0</v>
@@ -5867,7 +5864,7 @@
         <v>0</v>
       </c>
       <c r="E210">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F210">
         <v>2528</v>
@@ -5904,7 +5901,7 @@
         <v>218</v>
       </c>
       <c r="B212">
-        <v>2628</v>
+        <v>2658</v>
       </c>
       <c r="C212">
         <v>0</v>
@@ -5916,7 +5913,7 @@
         <v>14</v>
       </c>
       <c r="F212">
-        <v>2614</v>
+        <v>2644</v>
       </c>
       <c r="G212" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
update bulan 5 oktober 2026
</commit_message>
<xml_diff>
--- a/data/processed/rekap_qc.xlsx
+++ b/data/processed/rekap_qc.xlsx
@@ -1896,7 +1896,7 @@
         <v>44</v>
       </c>
       <c r="B38">
-        <v>2590</v>
+        <v>2591</v>
       </c>
       <c r="C38">
         <v>0</v>
@@ -1908,7 +1908,7 @@
         <v>65</v>
       </c>
       <c r="F38">
-        <v>2525</v>
+        <v>2526</v>
       </c>
       <c r="G38" t="b">
         <v>1</v>
@@ -2014,7 +2014,7 @@
         <v>2552</v>
       </c>
       <c r="C43">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="D43">
         <v>0</v>
@@ -2023,7 +2023,7 @@
         <v>57</v>
       </c>
       <c r="F43">
-        <v>2929</v>
+        <v>2932</v>
       </c>
       <c r="G43" t="b">
         <v>1</v>
@@ -2152,7 +2152,7 @@
         <v>2543</v>
       </c>
       <c r="C49">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D49">
         <v>0</v>
@@ -2161,7 +2161,7 @@
         <v>13</v>
       </c>
       <c r="F49">
-        <v>2572</v>
+        <v>2575</v>
       </c>
       <c r="G49" t="b">
         <v>1</v>
@@ -2264,7 +2264,7 @@
         <v>60</v>
       </c>
       <c r="B54">
-        <v>2005</v>
+        <v>2006</v>
       </c>
       <c r="C54">
         <v>0</v>
@@ -2276,7 +2276,7 @@
         <v>165</v>
       </c>
       <c r="F54">
-        <v>1840</v>
+        <v>1841</v>
       </c>
       <c r="G54" t="b">
         <v>1</v>
@@ -2310,7 +2310,7 @@
         <v>62</v>
       </c>
       <c r="B56">
-        <v>2674</v>
+        <v>2675</v>
       </c>
       <c r="C56">
         <v>1</v>
@@ -2322,7 +2322,7 @@
         <v>146</v>
       </c>
       <c r="F56">
-        <v>2529</v>
+        <v>2530</v>
       </c>
       <c r="G56" t="b">
         <v>1</v>
@@ -2333,7 +2333,7 @@
         <v>63</v>
       </c>
       <c r="B57">
-        <v>2757</v>
+        <v>2758</v>
       </c>
       <c r="C57">
         <v>4</v>
@@ -2342,7 +2342,7 @@
         <v>0</v>
       </c>
       <c r="E57">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F57">
         <v>2535</v>
@@ -2356,7 +2356,7 @@
         <v>64</v>
       </c>
       <c r="B58">
-        <v>1910</v>
+        <v>1911</v>
       </c>
       <c r="C58">
         <v>1</v>
@@ -2365,7 +2365,7 @@
         <v>0</v>
       </c>
       <c r="E58">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F58">
         <v>1836</v>
@@ -2448,7 +2448,7 @@
         <v>68</v>
       </c>
       <c r="B62">
-        <v>2621</v>
+        <v>2622</v>
       </c>
       <c r="C62">
         <v>0</v>
@@ -2460,7 +2460,7 @@
         <v>89</v>
       </c>
       <c r="F62">
-        <v>2532</v>
+        <v>2533</v>
       </c>
       <c r="G62" t="b">
         <v>1</v>
@@ -2471,7 +2471,7 @@
         <v>69</v>
       </c>
       <c r="B63">
-        <v>2620</v>
+        <v>2621</v>
       </c>
       <c r="C63">
         <v>1</v>
@@ -2483,7 +2483,7 @@
         <v>90</v>
       </c>
       <c r="F63">
-        <v>2532</v>
+        <v>2533</v>
       </c>
       <c r="G63" t="b">
         <v>1</v>
@@ -2494,7 +2494,7 @@
         <v>70</v>
       </c>
       <c r="B64">
-        <v>2629</v>
+        <v>2630</v>
       </c>
       <c r="C64">
         <v>0</v>
@@ -2506,7 +2506,7 @@
         <v>97</v>
       </c>
       <c r="F64">
-        <v>2533</v>
+        <v>2534</v>
       </c>
       <c r="G64" t="b">
         <v>1</v>
@@ -2517,7 +2517,7 @@
         <v>71</v>
       </c>
       <c r="B65">
-        <v>2621</v>
+        <v>2622</v>
       </c>
       <c r="C65">
         <v>0</v>
@@ -2529,7 +2529,7 @@
         <v>90</v>
       </c>
       <c r="F65">
-        <v>2531</v>
+        <v>2532</v>
       </c>
       <c r="G65" t="b">
         <v>1</v>
@@ -2540,7 +2540,7 @@
         <v>72</v>
       </c>
       <c r="B66">
-        <v>2628</v>
+        <v>2629</v>
       </c>
       <c r="C66">
         <v>2</v>
@@ -2552,7 +2552,7 @@
         <v>101</v>
       </c>
       <c r="F66">
-        <v>2532</v>
+        <v>2533</v>
       </c>
       <c r="G66" t="b">
         <v>1</v>
@@ -2563,7 +2563,7 @@
         <v>73</v>
       </c>
       <c r="B67">
-        <v>2619</v>
+        <v>2620</v>
       </c>
       <c r="C67">
         <v>1</v>
@@ -2575,7 +2575,7 @@
         <v>88</v>
       </c>
       <c r="F67">
-        <v>2532</v>
+        <v>2533</v>
       </c>
       <c r="G67" t="b">
         <v>1</v>
@@ -2586,7 +2586,7 @@
         <v>74</v>
       </c>
       <c r="B68">
-        <v>2624</v>
+        <v>2625</v>
       </c>
       <c r="C68">
         <v>0</v>
@@ -2598,7 +2598,7 @@
         <v>93</v>
       </c>
       <c r="F68">
-        <v>2531</v>
+        <v>2532</v>
       </c>
       <c r="G68" t="b">
         <v>1</v>
@@ -2609,7 +2609,7 @@
         <v>75</v>
       </c>
       <c r="B69">
-        <v>2624</v>
+        <v>2625</v>
       </c>
       <c r="C69">
         <v>0</v>
@@ -2621,7 +2621,7 @@
         <v>92</v>
       </c>
       <c r="F69">
-        <v>2532</v>
+        <v>2533</v>
       </c>
       <c r="G69" t="b">
         <v>1</v>
@@ -2632,7 +2632,7 @@
         <v>76</v>
       </c>
       <c r="B70">
-        <v>2628</v>
+        <v>2629</v>
       </c>
       <c r="C70">
         <v>1</v>
@@ -2644,7 +2644,7 @@
         <v>98</v>
       </c>
       <c r="F70">
-        <v>2532</v>
+        <v>2533</v>
       </c>
       <c r="G70" t="b">
         <v>1</v>
@@ -2655,7 +2655,7 @@
         <v>77</v>
       </c>
       <c r="B71">
-        <v>2622</v>
+        <v>2623</v>
       </c>
       <c r="C71">
         <v>0</v>
@@ -2667,7 +2667,7 @@
         <v>90</v>
       </c>
       <c r="F71">
-        <v>2532</v>
+        <v>2533</v>
       </c>
       <c r="G71" t="b">
         <v>1</v>
@@ -2678,7 +2678,7 @@
         <v>78</v>
       </c>
       <c r="B72">
-        <v>2624</v>
+        <v>2625</v>
       </c>
       <c r="C72">
         <v>3</v>
@@ -2690,7 +2690,7 @@
         <v>97</v>
       </c>
       <c r="F72">
-        <v>2531</v>
+        <v>2532</v>
       </c>
       <c r="G72" t="b">
         <v>1</v>
@@ -2701,7 +2701,7 @@
         <v>79</v>
       </c>
       <c r="B73">
-        <v>2751</v>
+        <v>2753</v>
       </c>
       <c r="C73">
         <v>6</v>
@@ -2710,10 +2710,10 @@
         <v>0</v>
       </c>
       <c r="E73">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F73">
-        <v>2559</v>
+        <v>2560</v>
       </c>
       <c r="G73" t="b">
         <v>1</v>
@@ -2747,7 +2747,7 @@
         <v>81</v>
       </c>
       <c r="B75">
-        <v>2847</v>
+        <v>2850</v>
       </c>
       <c r="C75">
         <v>6</v>
@@ -2759,7 +2759,7 @@
         <v>217</v>
       </c>
       <c r="F75">
-        <v>2637</v>
+        <v>2640</v>
       </c>
       <c r="G75" t="b">
         <v>1</v>
@@ -2770,7 +2770,7 @@
         <v>82</v>
       </c>
       <c r="B76">
-        <v>2864</v>
+        <v>2867</v>
       </c>
       <c r="C76">
         <v>12</v>
@@ -2782,7 +2782,7 @@
         <v>195</v>
       </c>
       <c r="F76">
-        <v>2683</v>
+        <v>2686</v>
       </c>
       <c r="G76" t="b">
         <v>1</v>
@@ -2793,7 +2793,7 @@
         <v>83</v>
       </c>
       <c r="B77">
-        <v>2855</v>
+        <v>2858</v>
       </c>
       <c r="C77">
         <v>5</v>
@@ -2805,7 +2805,7 @@
         <v>206</v>
       </c>
       <c r="F77">
-        <v>2654</v>
+        <v>2657</v>
       </c>
       <c r="G77" t="b">
         <v>1</v>
@@ -2816,7 +2816,7 @@
         <v>84</v>
       </c>
       <c r="B78">
-        <v>2747</v>
+        <v>2749</v>
       </c>
       <c r="C78">
         <v>0</v>
@@ -2825,10 +2825,10 @@
         <v>1</v>
       </c>
       <c r="E78">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F78">
-        <v>2558</v>
+        <v>2559</v>
       </c>
       <c r="G78" t="b">
         <v>1</v>
@@ -2839,7 +2839,7 @@
         <v>85</v>
       </c>
       <c r="B79">
-        <v>2844</v>
+        <v>2847</v>
       </c>
       <c r="C79">
         <v>0</v>
@@ -2851,7 +2851,7 @@
         <v>193</v>
       </c>
       <c r="F79">
-        <v>2652</v>
+        <v>2655</v>
       </c>
       <c r="G79" t="b">
         <v>1</v>
@@ -2885,7 +2885,7 @@
         <v>87</v>
       </c>
       <c r="B81">
-        <v>2846</v>
+        <v>2849</v>
       </c>
       <c r="C81">
         <v>1</v>
@@ -2897,7 +2897,7 @@
         <v>212</v>
       </c>
       <c r="F81">
-        <v>2635</v>
+        <v>2638</v>
       </c>
       <c r="G81" t="b">
         <v>1</v>
@@ -2908,7 +2908,7 @@
         <v>88</v>
       </c>
       <c r="B82">
-        <v>2867</v>
+        <v>2870</v>
       </c>
       <c r="C82">
         <v>3</v>
@@ -2920,7 +2920,7 @@
         <v>238</v>
       </c>
       <c r="F82">
-        <v>2633</v>
+        <v>2636</v>
       </c>
       <c r="G82" t="b">
         <v>1</v>
@@ -3138,7 +3138,7 @@
         <v>98</v>
       </c>
       <c r="B92">
-        <v>2583</v>
+        <v>2584</v>
       </c>
       <c r="C92">
         <v>1</v>
@@ -3150,7 +3150,7 @@
         <v>56</v>
       </c>
       <c r="F92">
-        <v>2528</v>
+        <v>2529</v>
       </c>
       <c r="G92" t="b">
         <v>1</v>
@@ -3161,7 +3161,7 @@
         <v>99</v>
       </c>
       <c r="B93">
-        <v>2586</v>
+        <v>2587</v>
       </c>
       <c r="C93">
         <v>0</v>
@@ -3173,7 +3173,7 @@
         <v>58</v>
       </c>
       <c r="F93">
-        <v>2528</v>
+        <v>2529</v>
       </c>
       <c r="G93" t="b">
         <v>1</v>
@@ -3184,7 +3184,7 @@
         <v>100</v>
       </c>
       <c r="B94">
-        <v>2585</v>
+        <v>2586</v>
       </c>
       <c r="C94">
         <v>8</v>
@@ -3196,7 +3196,7 @@
         <v>65</v>
       </c>
       <c r="F94">
-        <v>2528</v>
+        <v>2529</v>
       </c>
       <c r="G94" t="b">
         <v>1</v>
@@ -3207,7 +3207,7 @@
         <v>101</v>
       </c>
       <c r="B95">
-        <v>2580</v>
+        <v>2581</v>
       </c>
       <c r="C95">
         <v>5</v>
@@ -3219,7 +3219,7 @@
         <v>57</v>
       </c>
       <c r="F95">
-        <v>2528</v>
+        <v>2529</v>
       </c>
       <c r="G95" t="b">
         <v>1</v>
@@ -3230,7 +3230,7 @@
         <v>102</v>
       </c>
       <c r="B96">
-        <v>2582</v>
+        <v>2583</v>
       </c>
       <c r="C96">
         <v>1</v>
@@ -3242,7 +3242,7 @@
         <v>55</v>
       </c>
       <c r="F96">
-        <v>2528</v>
+        <v>2529</v>
       </c>
       <c r="G96" t="b">
         <v>1</v>
@@ -3253,7 +3253,7 @@
         <v>103</v>
       </c>
       <c r="B97">
-        <v>2584</v>
+        <v>2585</v>
       </c>
       <c r="C97">
         <v>7</v>
@@ -3265,7 +3265,7 @@
         <v>81</v>
       </c>
       <c r="F97">
-        <v>2528</v>
+        <v>2529</v>
       </c>
       <c r="G97" t="b">
         <v>1</v>
@@ -3276,7 +3276,7 @@
         <v>104</v>
       </c>
       <c r="B98">
-        <v>2582</v>
+        <v>2583</v>
       </c>
       <c r="C98">
         <v>15</v>
@@ -3288,7 +3288,7 @@
         <v>69</v>
       </c>
       <c r="F98">
-        <v>2528</v>
+        <v>2529</v>
       </c>
       <c r="G98" t="b">
         <v>1</v>
@@ -3299,7 +3299,7 @@
         <v>105</v>
       </c>
       <c r="B99">
-        <v>2584</v>
+        <v>2585</v>
       </c>
       <c r="C99">
         <v>1</v>
@@ -3311,7 +3311,7 @@
         <v>59</v>
       </c>
       <c r="F99">
-        <v>2529</v>
+        <v>2530</v>
       </c>
       <c r="G99" t="b">
         <v>1</v>
@@ -3322,7 +3322,7 @@
         <v>106</v>
       </c>
       <c r="B100">
-        <v>2585</v>
+        <v>2586</v>
       </c>
       <c r="C100">
         <v>0</v>
@@ -3334,7 +3334,7 @@
         <v>57</v>
       </c>
       <c r="F100">
-        <v>2528</v>
+        <v>2529</v>
       </c>
       <c r="G100" t="b">
         <v>1</v>
@@ -3368,7 +3368,7 @@
         <v>108</v>
       </c>
       <c r="B102">
-        <v>2589</v>
+        <v>2590</v>
       </c>
       <c r="C102">
         <v>1</v>
@@ -3380,7 +3380,7 @@
         <v>62</v>
       </c>
       <c r="F102">
-        <v>2528</v>
+        <v>2529</v>
       </c>
       <c r="G102" t="b">
         <v>1</v>
@@ -3391,7 +3391,7 @@
         <v>109</v>
       </c>
       <c r="B103">
-        <v>2589</v>
+        <v>2590</v>
       </c>
       <c r="C103">
         <v>0</v>
@@ -3403,7 +3403,7 @@
         <v>62</v>
       </c>
       <c r="F103">
-        <v>2528</v>
+        <v>2529</v>
       </c>
       <c r="G103" t="b">
         <v>1</v>
@@ -3414,7 +3414,7 @@
         <v>110</v>
       </c>
       <c r="B104">
-        <v>2626</v>
+        <v>2628</v>
       </c>
       <c r="C104">
         <v>1</v>
@@ -3423,10 +3423,10 @@
         <v>2</v>
       </c>
       <c r="E104">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F104">
-        <v>2542</v>
+        <v>2543</v>
       </c>
       <c r="G104" t="b">
         <v>1</v>
@@ -3437,7 +3437,7 @@
         <v>111</v>
       </c>
       <c r="B105">
-        <v>2623</v>
+        <v>2625</v>
       </c>
       <c r="C105">
         <v>0</v>
@@ -3446,10 +3446,10 @@
         <v>4</v>
       </c>
       <c r="E105">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F105">
-        <v>2542</v>
+        <v>2543</v>
       </c>
       <c r="G105" t="b">
         <v>1</v>
@@ -3460,7 +3460,7 @@
         <v>112</v>
       </c>
       <c r="B106">
-        <v>2620</v>
+        <v>2622</v>
       </c>
       <c r="C106">
         <v>0</v>
@@ -3469,10 +3469,10 @@
         <v>4</v>
       </c>
       <c r="E106">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F106">
-        <v>2542</v>
+        <v>2543</v>
       </c>
       <c r="G106" t="b">
         <v>1</v>
@@ -3483,7 +3483,7 @@
         <v>113</v>
       </c>
       <c r="B107">
-        <v>2623</v>
+        <v>2625</v>
       </c>
       <c r="C107">
         <v>1</v>
@@ -3492,10 +3492,10 @@
         <v>22</v>
       </c>
       <c r="E107">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F107">
-        <v>2542</v>
+        <v>2543</v>
       </c>
       <c r="G107" t="b">
         <v>1</v>
@@ -3506,7 +3506,7 @@
         <v>114</v>
       </c>
       <c r="B108">
-        <v>2618</v>
+        <v>2619</v>
       </c>
       <c r="C108">
         <v>0</v>
@@ -3515,7 +3515,7 @@
         <v>0</v>
       </c>
       <c r="E108">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F108">
         <v>2542</v>
@@ -3529,7 +3529,7 @@
         <v>115</v>
       </c>
       <c r="B109">
-        <v>2622</v>
+        <v>2624</v>
       </c>
       <c r="C109">
         <v>0</v>
@@ -3538,10 +3538,10 @@
         <v>27</v>
       </c>
       <c r="E109">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F109">
-        <v>2542</v>
+        <v>2543</v>
       </c>
       <c r="G109" t="b">
         <v>1</v>
@@ -3552,7 +3552,7 @@
         <v>116</v>
       </c>
       <c r="B110">
-        <v>2621</v>
+        <v>2623</v>
       </c>
       <c r="C110">
         <v>4</v>
@@ -3561,10 +3561,10 @@
         <v>1</v>
       </c>
       <c r="E110">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F110">
-        <v>2542</v>
+        <v>2543</v>
       </c>
       <c r="G110" t="b">
         <v>1</v>
@@ -3575,7 +3575,7 @@
         <v>117</v>
       </c>
       <c r="B111">
-        <v>2624</v>
+        <v>2626</v>
       </c>
       <c r="C111">
         <v>0</v>
@@ -3584,10 +3584,10 @@
         <v>4</v>
       </c>
       <c r="E111">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F111">
-        <v>2542</v>
+        <v>2543</v>
       </c>
       <c r="G111" t="b">
         <v>1</v>
@@ -3598,7 +3598,7 @@
         <v>118</v>
       </c>
       <c r="B112">
-        <v>2619</v>
+        <v>2621</v>
       </c>
       <c r="C112">
         <v>3</v>
@@ -3607,10 +3607,10 @@
         <v>0</v>
       </c>
       <c r="E112">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F112">
-        <v>2542</v>
+        <v>2543</v>
       </c>
       <c r="G112" t="b">
         <v>1</v>
@@ -3621,7 +3621,7 @@
         <v>119</v>
       </c>
       <c r="B113">
-        <v>2604</v>
+        <v>2605</v>
       </c>
       <c r="C113">
         <v>0</v>
@@ -3630,7 +3630,7 @@
         <v>2</v>
       </c>
       <c r="E113">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F113">
         <v>2530</v>
@@ -3644,7 +3644,7 @@
         <v>120</v>
       </c>
       <c r="B114">
-        <v>2645</v>
+        <v>2646</v>
       </c>
       <c r="C114">
         <v>1</v>
@@ -3656,7 +3656,7 @@
         <v>111</v>
       </c>
       <c r="F114">
-        <v>2535</v>
+        <v>2536</v>
       </c>
       <c r="G114" t="b">
         <v>1</v>
@@ -3667,7 +3667,7 @@
         <v>121</v>
       </c>
       <c r="B115">
-        <v>2634</v>
+        <v>2635</v>
       </c>
       <c r="C115">
         <v>0</v>
@@ -3679,7 +3679,7 @@
         <v>105</v>
       </c>
       <c r="F115">
-        <v>2529</v>
+        <v>2530</v>
       </c>
       <c r="G115" t="b">
         <v>1</v>
@@ -3874,7 +3874,7 @@
         <v>130</v>
       </c>
       <c r="B124">
-        <v>2641</v>
+        <v>2642</v>
       </c>
       <c r="C124">
         <v>1</v>
@@ -3886,7 +3886,7 @@
         <v>113</v>
       </c>
       <c r="F124">
-        <v>2529</v>
+        <v>2530</v>
       </c>
       <c r="G124" t="b">
         <v>1</v>
@@ -4012,7 +4012,7 @@
         <v>136</v>
       </c>
       <c r="B130">
-        <v>2635</v>
+        <v>2636</v>
       </c>
       <c r="C130">
         <v>0</v>
@@ -4024,7 +4024,7 @@
         <v>110</v>
       </c>
       <c r="F130">
-        <v>2525</v>
+        <v>2526</v>
       </c>
       <c r="G130" t="b">
         <v>1</v>
@@ -4035,7 +4035,7 @@
         <v>137</v>
       </c>
       <c r="B131">
-        <v>2635</v>
+        <v>2636</v>
       </c>
       <c r="C131">
         <v>1</v>
@@ -4047,7 +4047,7 @@
         <v>107</v>
       </c>
       <c r="F131">
-        <v>2529</v>
+        <v>2530</v>
       </c>
       <c r="G131" t="b">
         <v>1</v>
@@ -4104,7 +4104,7 @@
         <v>140</v>
       </c>
       <c r="B134">
-        <v>2637</v>
+        <v>2638</v>
       </c>
       <c r="C134">
         <v>0</v>
@@ -4116,7 +4116,7 @@
         <v>109</v>
       </c>
       <c r="F134">
-        <v>2529</v>
+        <v>2530</v>
       </c>
       <c r="G134" t="b">
         <v>1</v>
@@ -4265,7 +4265,7 @@
         <v>147</v>
       </c>
       <c r="B141">
-        <v>2720</v>
+        <v>2723</v>
       </c>
       <c r="C141">
         <v>0</v>
@@ -4277,7 +4277,7 @@
         <v>188</v>
       </c>
       <c r="F141">
-        <v>2532</v>
+        <v>2535</v>
       </c>
       <c r="G141" t="b">
         <v>1</v>
@@ -4357,7 +4357,7 @@
         <v>151</v>
       </c>
       <c r="B145">
-        <v>2948</v>
+        <v>2949</v>
       </c>
       <c r="C145">
         <v>0</v>
@@ -4366,7 +4366,7 @@
         <v>0</v>
       </c>
       <c r="E145">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F145">
         <v>2676</v>
@@ -4412,10 +4412,10 @@
         <v>0</v>
       </c>
       <c r="E147">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F147">
-        <v>2529</v>
+        <v>2528</v>
       </c>
       <c r="G147" t="b">
         <v>1</v>
@@ -4426,7 +4426,7 @@
         <v>154</v>
       </c>
       <c r="B148">
-        <v>2843</v>
+        <v>2846</v>
       </c>
       <c r="C148">
         <v>1</v>
@@ -4438,7 +4438,7 @@
         <v>306</v>
       </c>
       <c r="F148">
-        <v>2539</v>
+        <v>2542</v>
       </c>
       <c r="G148" t="b">
         <v>1</v>
@@ -4449,7 +4449,7 @@
         <v>155</v>
       </c>
       <c r="B149">
-        <v>2959</v>
+        <v>2960</v>
       </c>
       <c r="C149">
         <v>0</v>
@@ -4461,7 +4461,7 @@
         <v>194</v>
       </c>
       <c r="F149">
-        <v>2765</v>
+        <v>2766</v>
       </c>
       <c r="G149" t="b">
         <v>1</v>
@@ -4472,7 +4472,7 @@
         <v>156</v>
       </c>
       <c r="B150">
-        <v>2760</v>
+        <v>2761</v>
       </c>
       <c r="C150">
         <v>0</v>
@@ -4484,7 +4484,7 @@
         <v>232</v>
       </c>
       <c r="F150">
-        <v>2528</v>
+        <v>2529</v>
       </c>
       <c r="G150" t="b">
         <v>1</v>
@@ -5007,10 +5007,10 @@
         <v>0</v>
       </c>
       <c r="D173">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E173">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F173">
         <v>2528</v>
@@ -5024,7 +5024,7 @@
         <v>180</v>
       </c>
       <c r="B174">
-        <v>2928</v>
+        <v>2930</v>
       </c>
       <c r="C174">
         <v>0</v>
@@ -5033,10 +5033,10 @@
         <v>0</v>
       </c>
       <c r="E174">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="F174">
-        <v>2591</v>
+        <v>2587</v>
       </c>
       <c r="G174" t="b">
         <v>1</v>
@@ -5093,7 +5093,7 @@
         <v>183</v>
       </c>
       <c r="B177">
-        <v>2719</v>
+        <v>2722</v>
       </c>
       <c r="C177">
         <v>0</v>
@@ -5105,7 +5105,7 @@
         <v>35</v>
       </c>
       <c r="F177">
-        <v>2684</v>
+        <v>2687</v>
       </c>
       <c r="G177" t="b">
         <v>1</v>
@@ -5116,7 +5116,7 @@
         <v>184</v>
       </c>
       <c r="B178">
-        <v>2946</v>
+        <v>2947</v>
       </c>
       <c r="C178">
         <v>0</v>
@@ -5128,7 +5128,7 @@
         <v>196</v>
       </c>
       <c r="F178">
-        <v>2751</v>
+        <v>2752</v>
       </c>
       <c r="G178" t="b">
         <v>1</v>
@@ -5139,7 +5139,7 @@
         <v>185</v>
       </c>
       <c r="B179">
-        <v>2950</v>
+        <v>2951</v>
       </c>
       <c r="C179">
         <v>0</v>
@@ -5148,7 +5148,7 @@
         <v>0</v>
       </c>
       <c r="E179">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F179">
         <v>2603</v>
@@ -5162,7 +5162,7 @@
         <v>186</v>
       </c>
       <c r="B180">
-        <v>2928</v>
+        <v>2929</v>
       </c>
       <c r="C180">
         <v>1</v>
@@ -5171,7 +5171,7 @@
         <v>2</v>
       </c>
       <c r="E180">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F180">
         <v>2609</v>
@@ -5185,7 +5185,7 @@
         <v>187</v>
       </c>
       <c r="B181">
-        <v>2942</v>
+        <v>2943</v>
       </c>
       <c r="C181">
         <v>0</v>
@@ -5194,7 +5194,7 @@
         <v>0</v>
       </c>
       <c r="E181">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F181">
         <v>2603</v>
@@ -5208,7 +5208,7 @@
         <v>188</v>
       </c>
       <c r="B182">
-        <v>2947</v>
+        <v>2948</v>
       </c>
       <c r="C182">
         <v>0</v>
@@ -5217,7 +5217,7 @@
         <v>1</v>
       </c>
       <c r="E182">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="F182">
         <v>2606</v>
@@ -5231,7 +5231,7 @@
         <v>189</v>
       </c>
       <c r="B183">
-        <v>2962</v>
+        <v>2963</v>
       </c>
       <c r="C183">
         <v>0</v>
@@ -5240,7 +5240,7 @@
         <v>0</v>
       </c>
       <c r="E183">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F183">
         <v>2602</v>
@@ -5254,7 +5254,7 @@
         <v>190</v>
       </c>
       <c r="B184">
-        <v>2927</v>
+        <v>2928</v>
       </c>
       <c r="C184">
         <v>0</v>
@@ -5263,7 +5263,7 @@
         <v>0</v>
       </c>
       <c r="E184">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F184">
         <v>2567</v>
@@ -5484,7 +5484,7 @@
         <v>200</v>
       </c>
       <c r="B194">
-        <v>2625</v>
+        <v>2626</v>
       </c>
       <c r="C194">
         <v>1</v>
@@ -5493,10 +5493,10 @@
         <v>0</v>
       </c>
       <c r="E194">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="F194">
-        <v>2541</v>
+        <v>2539</v>
       </c>
       <c r="G194" t="b">
         <v>1</v>
@@ -5553,7 +5553,7 @@
         <v>203</v>
       </c>
       <c r="B197">
-        <v>1880</v>
+        <v>1881</v>
       </c>
       <c r="C197">
         <v>0</v>
@@ -5565,7 +5565,7 @@
         <v>49</v>
       </c>
       <c r="F197">
-        <v>1831</v>
+        <v>1832</v>
       </c>
       <c r="G197" t="b">
         <v>1</v>
@@ -5622,7 +5622,7 @@
         <v>206</v>
       </c>
       <c r="B200">
-        <v>3195</v>
+        <v>3198</v>
       </c>
       <c r="C200">
         <v>0</v>
@@ -5634,7 +5634,7 @@
         <v>0</v>
       </c>
       <c r="F200">
-        <v>3195</v>
+        <v>3198</v>
       </c>
       <c r="G200" t="b">
         <v>1</v>
@@ -5645,7 +5645,7 @@
         <v>207</v>
       </c>
       <c r="B201">
-        <v>3195</v>
+        <v>3198</v>
       </c>
       <c r="C201">
         <v>1</v>
@@ -5657,7 +5657,7 @@
         <v>0</v>
       </c>
       <c r="F201">
-        <v>3196</v>
+        <v>3199</v>
       </c>
       <c r="G201" t="b">
         <v>0</v>
@@ -5671,7 +5671,7 @@
         <v>208</v>
       </c>
       <c r="B202">
-        <v>2899</v>
+        <v>2902</v>
       </c>
       <c r="C202">
         <v>0</v>
@@ -5683,7 +5683,7 @@
         <v>299</v>
       </c>
       <c r="F202">
-        <v>2600</v>
+        <v>2603</v>
       </c>
       <c r="G202" t="b">
         <v>1</v>
@@ -5901,7 +5901,7 @@
         <v>218</v>
       </c>
       <c r="B212">
-        <v>2658</v>
+        <v>2661</v>
       </c>
       <c r="C212">
         <v>0</v>
@@ -5913,7 +5913,7 @@
         <v>14</v>
       </c>
       <c r="F212">
-        <v>2644</v>
+        <v>2647</v>
       </c>
       <c r="G212" t="b">
         <v>1</v>

</xml_diff>